<commit_message>
Laporan QA sebelum/sesudah dalam format Excel
Satu berkas, empat lembar: Ringkasan (temuan per tingkat dan per area, plus
jumlah uji sebelum dan sesudah), Audit tim (34 temuan), Skenario kanvas (63
skenario yang dijalankan lewat Chrome sungguhan, ditandai LOLOS atau
DIPERBAIKI), dan Audit kanvas (5 temuan).

Tiap baris temuan memuat perilaku SEBELUM dan SESUDAH berdampingan, beserta
angka sungguhan dari pengujiannya — bukan ringkasan, melainkan keluaran yang
benar-benar tercatat saat diuji.

Berkasnya sendiri tidak ikut repo: ia dibuat ulang dari data pengujian, dan
menyimpan biner yang berubah tiap kali dijalankan cuma membuat riwayat sulit
dibaca.
</commit_message>
<xml_diff>
--- a/label-apps/laporan/QA-higo-label.xlsx
+++ b/label-apps/laporan/QA-higo-label.xlsx
@@ -9,9 +9,13 @@
   <sheets>
     <sheet name="Ringkasan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Audit tim" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Skenario kanvas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Audit kanvas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Audit tim'!$A$2:$J$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Skenario kanvas'!$A$2:$C$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit kanvas'!$A$2:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -553,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -649,13 +653,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -671,13 +675,13 @@
         <v>10</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>0</v>
@@ -693,13 +697,13 @@
         <v>10</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -737,13 +741,13 @@
         <v>34</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>0</v>
@@ -867,89 +871,141 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C24" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Urungkan</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>PENGUJIAN OTOMATIS</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Rangkaian</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Sebelum</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Sesudah</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B32" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C32" s="6" t="n">
         <v>376</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>uji peramban (kanvas)</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n">
+      <c r="B33" s="6" t="n">
         <v>162</v>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C33" s="6" t="n">
         <v>170</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>sapuan dev</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B34" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C34" s="6" t="n">
         <v>48</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>uji salin</t>
         </is>
       </c>
-      <c r="B31" s="6" t="n">
+      <c r="B35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C35" s="6" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2748,4 +2804,1478 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C66"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Seluruh skenario yang dijalankan lewat Chrome sungguhan (CDP) terhadap server dev. LOLOS = benar sejak awal. DIPERBAIKI = gagal saat diuji, lalu diperbaiki dan diuji ulang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Bagian</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Skenario</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Hasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>R memilih mode kotak; seret menghasilkan satu rectangle 2 titik</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Poligon: 4 klik lalu Enter menutup jadi polygon 4 titik</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Ctrl+Z saat menggambar mencabut satu titik draft, bukan objek jadi</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Esc membuang draft yang sedang digambar</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Lingkaran (seret dari pusat) menghasilkan circle</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Garis (dua klik) menghasilkan line</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Titik (satu klik) menghasilkan point</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Alat gambar</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Garis patah: 3 klik lalu Enter menghasilkan linestrip 3 titik</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Mode sunting</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>V lalu klik memilih objek (S.sel)</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Mode sunting</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Menyeret objek benar-benar menggeser koordinatnya</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Mode sunting</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Delete menghapus objek terpilih</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Urungkan</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Ctrl+Z mundur satu langkah tiap kali (2 -&gt; 1 -&gt; 0)</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Urungkan</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Ctrl+Y mengulang yang barusan diurungkan</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Urungkan</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Ctrl+Shift+Z juga mengulang</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Urungkan</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Perubahan baru memutus cabang redo</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Grup</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>G memberi group_id yang sama ke objek terpilih</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Grup</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>U melepas grup</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Zoom &amp; geser</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Koordinat objek tidak berubah sesudah zoom ekstrem + muat ke layar</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Q memilih mode +Point</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Klik pada objek menghasilkan pratinjau (8 titik)</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Prompt tercatat satu titik</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>C membersihkan prompt dan pratinjau</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>F membuka dialog kelas</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Kotak kelas KOSONG, bukan berisi huruf 'f'</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Fokus otomatis di kotak kelas</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Nama kelas ' ' ditolak: 'Nama kelas belum diisi'</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Nama kelas 'a' ditolak: minimal dua karakter</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Nama kelas ' botol' dipangkas dan diterima</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Objek tersimpan dengan kelas yang diketik</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Group ID bukan angka ditolak</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Group ID angka diterima dan tersimpan</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Batal tidak menambah objek</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Daftar kelas menampilkan SELURUH kelas walau kotak terisi</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Mengetik menyaring daftar</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>Deteksi teks</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Teks kosong ditolak dengan pesan</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Simpan menulis berkas anotasi ke disk</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Kelas, jenis, dan titik bulat-balik (poligon ditulis tertutup)</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>group_id bulat-balik</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>flags bulat-balik</t>
+        </is>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Catatan objek bulat-balik</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Objek terbaca lagi sesudah muat ulang</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Simpan ulang tanpa perubahan tidak merusak berkas (3 putaran)</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Bentuk bertitik kurang tidak diam-diam menjadikan gambar latar</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>OBJECTS menghitung dan menampilkan barisnya</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>FLAGS: tambah flag gambar lewat Enter</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>LABELS: tambah kelas baru lewat Enter</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>SETELAN: kecerahan berubah</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>SETELAN: kembalikan normal</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>FILES memuat seluruh daftar berkas</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>D pindah ke gambar berikutnya</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>A kembali ke gambar sebelumnya</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Perubahan menandai sesi kotor (menahan navigasi)</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>Hak per gambar</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Pelabel boleh menyimpan gambar jatahnya</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Hak per gambar</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Pelabel ditolak pada gambar yang bukan jatahnya</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>Hak per gambar</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Berkas gambar orang lain tidak tertulis</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Hak per gambar</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Kanvas gambar orang lain dibuka hanya-baca (BACA_SAJA)</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Poligon yang seluruh titiknya sama ditandai 'perlu dicek'</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>Bentuk raksasa melebihi frame dikurung dan ditandai</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Bentuk tanpa kelas ditolak dengan pesan</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Gambar dengan anotasi rusak tetap membuka kanvas</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>Kerusakan berkas disebutkan di layar</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Berkas rusak disisihkan, bukan ditimpa</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>Tandai latar</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Gambar kosong bisa ditandai latar</t>
+        </is>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>Tandai latar</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>Gambar berisi objek ditolak</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:C66"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Audit halaman kanvas pelabelan (/label): alat gambar, mode sunting, SAM dan deteksi teks, dialog kelas, penyimpanan, panel kanan, dan navigasi. Tiga agen QA, 3 September 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Tingkat</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Temuan</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>SEBELUM — perilaku yang salah</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>SESUDAH — perilaku sekarang</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Bukti (angka sungguhan)</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Berkas</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>Dikunci uji</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Simpan</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>TINGGI</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Bentuk bertitik kurang dibuang diam-diam, gambarnya jadi sampel negatif</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Bentuk yang titiknya di bawah minimum (poligon &lt;3, kotak/garis &lt;2) dibuang lewat `continue` tanpa dicatat. Kalau SELURUH bentuk terbuang, berkas ditulis dengan shapes kosong — dan berkas anotasi kosong adalah PENANDA LATAR. Balasannya ok:true. Orang menggambar sesuatu, menekan simpan, dan gambarnya diam-diam berubah jadi contoh negatif yang ikut dilatih.</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Kalau semua bentuk terbuang, permintaan ditolak dan berkas tidak ditulis sama sekali. Kalau sebagian terbuang, jumlahnya dilaporkan di balasan dan ditoast di layar.</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: {'ok': True, 'n': 0, 'sev': 'bg'}, berkas berisi shapes: [], gambar tampil di saringan Latar. Sesudah: {'ok': False, '1 bentuk dibuang karena titiknya kurang - Gambar tidak diubah.'}, berkas tidak dibuat.</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>app/routers/annotate.py:api_simpan</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>dibuktikan di dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>SEDANG</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Daftar kelas runtuh jadi satu baris justru saat dibutuhkan</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Kotak kelas terisi kelas terakhir (setelan 'Pertahankan label terakhir', menyala secara bawaan), dan gambarDaftar() menyaring memakai isi kotak itu. Akibatnya daftar kelas — satu-satunya tempat melihat pilihan yang ada — menyusut jadi satu entri persis ketika orang membukanya untuk memilih kelas yang LAIN.</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Daftar hanya disaring sesudah orang mengetik sendiri. Isi pra-isinya juga disorot, jadi mengetik langsung menggantinya tanpa perlu menghapus dulu.</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: S.kelas ['botol','kaleng','mlp'], dialog menampilkan ['kaleng'] saja. Sesudah: menampilkan ketiganya; mengetik 'bo' menyaring jadi ['botol'].</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>app/static/label.js:tanyaKelas</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>dibuktikan di dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Urungkan</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>SEDANG</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Tidak ada Ulangi sama sekali — 40 langkah mundur, nol maju</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>S.undo menyimpan 40 langkah, tetapi tidak ada jalan kembali. Satu Ctrl+Z yang kelewat berarti menggambar ulang dari awal, dan itu paling sering terjadi saat menggambar poligon berpuluh titik. Ctrl+Y dan Ctrl+Shift+Z tidak melakukan apa pun.</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Ditambahkan S.redo beserta fungsi ulangi(), terikat ke Ctrl+Y dan Ctrl+Shift+Z, dan dicatat di Panduan. Perubahan baru memutus cabang redo supaya Ctrl+Y tidak pernah melompat ke keadaan yang tidak pernah ada.</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: gambar 2 objek, urungkan 2x -&gt; 0, Ctrl+Y -&gt; tetap 0. Sesudah: Ctrl+Y -&gt; 1, Ctrl+Shift+Z -&gt; 1, dan sesudah menggambar baru Ctrl+Y tidak melompat.</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>app/static/label.js:ulangi</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>dibuktikan di dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Dialog kelas</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>RENDAH</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Pesan galat menjanjikan aturan yang tidak berlaku</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Pesannya berbunyi 'minimal dua karakter dan tidak boleh diawali spasi', padahal setuju() memangkas spasi lebih dulu sehingga ' botol' diterima dan tersimpan sebagai 'botol'.</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Perilakunya dipertahankan (memangkas itu ramah), tetapi kalimatnya tidak lagi menjanjikan aturan yang tidak dijalankan.</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: ' botol' diterima walau pesannya bilang tidak boleh. Sesudah: diterima, dan pesannya cuma menyebut aturan yang benar-benar berlaku.</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>app/static/label.js:namaKelasSah</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Kasus tepi</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>SEDANG</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Berkas anotasi rusak dibuka sebagai "siap" lalu ditimpa</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Berkas .json yang tidak bisa dibaca menghasilkan kanvas dengan nol objek dan status 'i2.jpg siap'. Tidak ada satu pun tanda di layar. Orang melabeli dari nol, menyimpan, dan berkas lamanya hilang — bersamanya satu-satunya kesempatan memperbaikinya dengan tangan. /markbg sudah menolak berkas rusak sejak awal; /api/simpan tidak.</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Kanvas menampilkan peringatan tetap di atas gambar, dan menyimpan menyisihkan berkas rusaknya jadi .json.rusak-&lt;cap waktu&gt; lebih dulu, bukan menimpanya.</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: status 'siap', issues [], berkas tertimpa. Sesudah: peringatan 'tidak bisa dibaca' tampil, dan folder berisi i2.json + i2.json.rusak-1788402084.</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>app/routers/annotate.py:selamatkan_rusak, label.html</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>tests/test_data.py</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J7"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Laporan QA diperbarui: 40 temuan, 85 skenario kanvas
</commit_message>
<xml_diff>
--- a/label-apps/laporan/QA-higo-label.xlsx
+++ b/label-apps/laporan/QA-higo-label.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Audit tim'!$A$2:$J$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Skenario kanvas'!$A$2:$C$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit kanvas'!$A$2:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Skenario kanvas'!$A$2:$C$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit kanvas'!$A$2:$J$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -653,13 +653,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -741,13 +741,13 @@
         <v>34</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>0</v>
@@ -933,79 +933,92 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Kerja bersamaan</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>PENGUJIAN OTOMATIS</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Rangkaian</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Sebelum</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Sesudah</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>pytest</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="n">
-        <v>331</v>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>376</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>uji peramban (kanvas)</t>
+          <t>pytest</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>162</v>
+        <v>331</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>170</v>
+        <v>376</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>sapuan dev</t>
+          <t>uji peramban (kanvas)</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>43</v>
+        <v>162</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>48</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
+          <t>sapuan dev</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
           <t>uji salin</t>
         </is>
       </c>
-      <c r="B35" s="6" t="n">
+      <c r="B36" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C36" s="6" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2812,7 +2825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3932,8 +3945,365 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>Undangan surel</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>Undangan email menghasilkan tautan untuk disalin</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>Undangan surel</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Balasannya tidak mengaku mengirim surel</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>Undangan surel</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Layarnya tidak menjanjikan surel otomatis</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>Tata letak YOLO</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Projek images/+labels/+data.yaml bisa dibuka</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>Tata letak YOLO</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>Kanvas memuat kelas resmi dari data.yaml</t>
+        </is>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>Tata letak YOLO</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>Menyimpan menulis kembali .txt dengan indeks kelas benar</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>Tata letak YOLO</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Cadangan .json menyimpan yang tidak muat di .txt</t>
+        </is>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>Tata letak YOLO</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>group_id dan catatan bertahan lewat cadangan</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>Tulis bersamaan</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>Empat penulisan serentak semuanya dijawab</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>Tulis bersamaan</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>Berkas tetap JSON sah dan utuh (tulis atomik)</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>Ganti model SAM</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>Dropdown memuat lima model</t>
+        </is>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>Ganti model SAM</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Ganti model menjalankan ulang SAM dan melaporkan hasilnya</t>
+        </is>
+      </c>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>Ganti model SAM</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Model baru menghasilkan pratinjau</t>
+        </is>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>Deteksi teks</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>Deteksi menjawab dengan objek berkelas</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>Pertahankan anotasi</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>Setelan bisa dinyalakan</t>
+        </is>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Pertahankan anotasi</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>Gambar berikutnya mewarisi anotasi sebelumnya</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>Pertahankan anotasi</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>Warisannya ikut tertulis ke disk</t>
+        </is>
+      </c>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>Pertahankan anotasi</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>Gambar yang sudah berisi TIDAK ditimpa</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>Dua tab</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>Berkas tetap sah sesudah dua tab menyimpan</t>
+        </is>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>Dua tab</t>
+        </is>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>Tulisan terakhir menang tanpa merusak berkas</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>Dua tab</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>Tab lama melihat isi terbaru sesudah dimuat ulang</t>
+        </is>
+      </c>
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:C66"/>
+  <autoFilter ref="A2:C87"/>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
@@ -3947,7 +4317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4271,8 +4641,58 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Kerja bersamaan</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>TINGGI</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Kanvas menampilkan anotasi versi lama, lalu menimpanya</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Isi projek dipindai sekali lalu dipakai dari ingatan sesi, dan halaman kanvas maupun halaman Lihat tidak pernah menyegarkannya. Dua orang pada gambar yang sama: yang satu membuka, yang lain menyimpan, lalu yang pertama menyimpan di atas dasar yang sudah usang — dan pekerjaan yang di antaranya hilang tanpa jejak.</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Kedua halaman menyegarkan diri lewat penanda perubahan per projek, sama seperti papan dan grid. Murah kalau tidak ada yang berubah: yang menaikkan penandanya cuma penulisan sungguhan.</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: tab A menyimpan 'dari-tab-A', tab B menyimpan 'dari-tab-B', tab A dimuat ulang masih menampilkan 'dari-tab-A'. Sesudah: menampilkan 'dari-tab-B'.</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>app/routers/annotate.py:halaman, review.py:view</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>tests/test_akses.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:J7"/>
+  <autoFilter ref="A2:J8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Laporan QA final: 42 temuan, 99 skenario
</commit_message>
<xml_diff>
--- a/label-apps/laporan/QA-higo-label.xlsx
+++ b/label-apps/laporan/QA-higo-label.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Audit tim'!$A$2:$J$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Skenario kanvas'!$A$2:$C$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit kanvas'!$A$2:$J$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Skenario kanvas'!$A$2:$C$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit kanvas'!$A$2:$J$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -653,13 +653,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -675,13 +675,13 @@
         <v>10</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>0</v>
@@ -741,13 +741,13 @@
         <v>34</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>0</v>
@@ -884,20 +884,20 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Dataset</t>
+          <t>Kinerja</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Simpan</t>
+          <t>Dataset</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
@@ -910,7 +910,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Urungkan</t>
+          <t>Simpan</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
@@ -923,7 +923,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Kasus tepi</t>
+          <t>Urungkan</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
@@ -936,7 +936,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Kerja bersamaan</t>
+          <t>Kasus tepi</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
@@ -946,79 +946,92 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Kerja bersamaan</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>PENGUJIAN OTOMATIS</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Rangkaian</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Sebelum</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Sesudah</t>
         </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>pytest</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>331</v>
-      </c>
-      <c r="C33" s="6" t="n">
-        <v>376</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>uji peramban (kanvas)</t>
+          <t>pytest</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>162</v>
+        <v>331</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>170</v>
+        <v>376</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>sapuan dev</t>
+          <t>uji peramban (kanvas)</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>43</v>
+        <v>162</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>48</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
+          <t>sapuan dev</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
           <t>uji salin</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n">
+      <c r="B37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C36" s="6" t="n">
+      <c r="C37" s="6" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2825,7 +2838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4302,8 +4315,246 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>Beban 8 pelabel</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>920-1280 operasi tanpa jeda, nol permintaan gagal</t>
+        </is>
+      </c>
+      <c r="C88" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>Beban 8 pelabel</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>Seluruh berkas anotasi tetap JSON yang sah</t>
+        </is>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>Beban 8 pelabel</t>
+        </is>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>Berkas tugas dan tag tetap sah dan lengkap</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>Beban 8 pelabel</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>Tidak ada gambar tercatat di dua job</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>Beban 8 pelabel</t>
+        </is>
+      </c>
+      <c r="B92" s="14" t="inlineStr">
+        <is>
+          <t>Tidak ada berkas sementara tertinggal</t>
+        </is>
+      </c>
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>Beban 8 pelabel</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>Papan tetap responsif walau ditulisi terus</t>
+        </is>
+      </c>
+      <c r="C93" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>Server mati</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>SIGKILL di tengah 1.140 penulisan: tidak ada berkas rusak</t>
+        </is>
+      </c>
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Server mati</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>Tidak ada berkas anotasi berukuran nol</t>
+        </is>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>Server mati</t>
+        </is>
+      </c>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>Tidak ada .tmp maupun .part tertinggal</t>
+        </is>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Server mati</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>Berkas tugas tetap terbaca</t>
+        </is>
+      </c>
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>Server mati</t>
+        </is>
+      </c>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t>Server bisa dinyalakan lagi</t>
+        </is>
+      </c>
+      <c r="C98" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="inlineStr">
+        <is>
+          <t>Server mati</t>
+        </is>
+      </c>
+      <c r="B99" s="14" t="inlineStr">
+        <is>
+          <t>Projek terbuka utuh dengan seluruh anotasinya</t>
+        </is>
+      </c>
+      <c r="C99" s="16" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>Kinerja</t>
+        </is>
+      </c>
+      <c r="B100" s="14" t="inlineStr">
+        <is>
+          <t>Telusur projek 11.319 gambar di bawah 100 ms</t>
+        </is>
+      </c>
+      <c r="C100" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>Kinerja</t>
+        </is>
+      </c>
+      <c r="B101" s="14" t="inlineStr">
+        <is>
+          <t>Hitungan gambar persis, bukan '≥' yang menyerah di tengah</t>
+        </is>
+      </c>
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t>DIPERBAIKI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:C87"/>
+  <autoFilter ref="A2:C101"/>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
@@ -4317,7 +4568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4691,8 +4942,108 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Kinerja</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>TINGGI</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Penyegaran sesi memindai ulang seluruh folder tiap ada yang menulis</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Perbaikan papan-yang-membeku dipasang dengan memindai ulang seluruh projek setiap kali penanda perubahan bergerak. Pada projek produksi terbesar sekali pindai 5,84 detik untuk 11.319 gambar — jadi satu tim yang sedang melabeli membuat SETIAP muat halaman menunggu enam detik. Regresi yang saya buat sendiri, dan baru ketahuan lewat uji beban.</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Yang dibaca ulang hanya gambar yang benar-benar berubah: penulisnya menyebutkan berkas mana. Riwayatnya dibatasi; sesi yang tertinggal lebih jauh memindai ulang seluruhnya.</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>Sebelum: papan 558 ms pada projek yang baru ditulisi. Sesudah: 34 ms.</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>app/session.py:segarkan, berubah_sejak</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>tests/test_data.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Kinerja</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>SEDANG</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Telusur folder mahal, dan hitungannya berhenti di tengah jalan</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>_survei dipanggil setiap halaman projek lewat konteks(). Pada projek 11.319 gambar ia memakan 542 ms — 276 ms di antaranya untuk anotasi_untuk yang men-stat tiap gambar sampai tiga kali hanya demi memilih sampul, ditambah satu stat per entri dari rglob. Batas 20.000 entri juga membuatnya menyerah di tengah: kartunya menyebut '≥10.187 gambar' untuk 11.319 yang sebenarnya, dan angka itu ikut ke lencana sidebar.</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Ditulis ulang memakai os.scandir dengan pasangan anotasi ditentukan dari telusur yang sama; batasnya dinaikkan ke 60.000. Tanpa simpanan — tidak ada kebenaran yang ditaruh di tempat kedua.</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>542 ms -&gt; 83 ms pada projek prod, 74 ms -&gt; 8 ms pada 476 gambar, versi.daftar 68 ms -&gt; 0,9 ms, dan angkanya kini persis 11.319 bukan '≥10.187'.</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>app/services/projek.py:_survei, versi.py:daftar</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>tests/test_projek.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:J8"/>
+  <autoFilter ref="A2:J10"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>

</xml_diff>